<commit_message>
Update to figures and docs
</commit_message>
<xml_diff>
--- a/docs/amps_prediction.xlsx
+++ b/docs/amps_prediction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luigui/Documents/amps_microbiome_2025/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4F4603-4A2F-854D-8002-8BBD54A0A938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588C9F4A-06DC-0B4F-8318-330394CB3A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="5" xr2:uid="{D0FE8B26-41E0-2A46-B2EA-AAB3A158C054}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="3" xr2:uid="{D0FE8B26-41E0-2A46-B2EA-AAB3A158C054}"/>
   </bookViews>
   <sheets>
     <sheet name="420_AMPs" sheetId="1" r:id="rId1"/>

</xml_diff>